<commit_message>
docs: integrate latest K8S evidence into v3.1.18 candidate
Sync K8S/ICR/SEC descriptions, WBS sources, schedule task wording and release package checksums. Preserve statuses, dates, AC history and prior snapshots. Record PR #3 merge and PR #2/#4 evidence while retaining pending review and runtime acceptance.
</commit_message>
<xml_diff>
--- a/wbs/FDS_v3.1.18_WBS_and_Gantt_v1.0.xlsx
+++ b/wbs/FDS_v3.1.18_WBS_and_Gantt_v1.0.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R59de15557d2a40d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R02f318c594b54eb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R133389d2406949a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rc6fea7b1f7584016"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R6a72812e68f84ecf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="Rc9345d8e43814cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R007f1f2aae214edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R028937b20bd648cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Ra654dbb8f62d440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R137a26d119ab4fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R2b78cea4860f46f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R02176cc0027a4d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R4b8617fd2af240c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R3b845c23c57a46c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R279c4388cc5a4e37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R31006a1b979b4f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R09d66d5b4d934e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R0014c28a50aa4e63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="38">
+  <x:dxfs count="39">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1000,6 +1000,17 @@
         <x:color rgb="FFB4233D"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFDE3E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB4233D"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE3E7"/>
         </x:patternFill>
@@ -1255,7 +1266,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbe51134b881f4031"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rae5a8ad124bb46de"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1285,7 +1296,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8d2e98215b35452d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3d52f5ad47624164"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1971,7 +1982,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3453ac8c19674810"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a2969211bc44256"/>
 </x:worksheet>
 </file>
 
@@ -2357,7 +2368,7 @@
         <x:v>09-11 CP1, 09-14 CP2/3·Worker, 09-15 NTP·Calico, 09-17 증적 인수를 조건부 목표로 둔다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R7" s="13" t="str">
-        <x:v>Baseline v3.1.18; Ticket Pack v3.1.18; GitHub #10 snapshot 2026-09-10T05:03:27Z; Issue #10 후속 2026-09-10T06:25:12Z; infra-kubernetes PR #3 @3309866766236bbdbe20b9e2ae1d8fd6f9233bcd; Fast Tracking 일정 권장안 2026-09-10 / 사용자 재편성 요청</x:v>
+        <x:v>Baseline/Ticket Pack v3.1.18; GitHub #10; K8S PR #2 097ddb5, #3 merge 7d44afc, #4 75d476e; audit/v3.1.18/k8s-intake-20260910.json</x:v>
       </x:c>
       <x:c r="S7" s="13" t="str">
         <x:f>IF(G7="Done","Done",IF(I7="",IF(F7="P1","Deferred P1","End TBD"),IF(I7&lt;'Executive Summary'!$B$4,"Overdue",IF(H7&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -2605,7 +2616,7 @@
         <x:v>09-21은 권장 Plan End이며 실제 종료일 확정이나 AC 완료가 아니다. 기존 End TBD 이력은 보존한다. CP→Worker·NTP·IF-16을 먼저, IF-06B·Negative/Reboot/Rollback·보호 인계를 후속 검증한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R11" s="13" t="str">
-        <x:v>Baseline v3.1.18; Ticket Pack v3.1.18; GitHub #14 snapshot 2026-09-10T05:03:39Z; Issue #14 후속 2026-09-10T06:25:25Z; infra-kubernetes PR #3 @3309866766236bbdbe20b9e2ae1d8fd6f9233bcd; Fast Tracking 일정 권장안 2026-09-10 / 사용자 재편성 요청</x:v>
+        <x:v>Baseline/Ticket Pack v3.1.18; GitHub #14; K8S PR #2 097ddb5, #3 merge 7d44afc, #4 75d476e; audit/v3.1.18/k8s-intake-20260910.json</x:v>
       </x:c>
       <x:c r="S11" s="13" t="str">
         <x:f>IF(G11="Done","Done",IF(I11="",IF(F11="P1","Deferred P1","End TBD"),IF(I11&lt;'Executive Summary'!$B$4,"Overdue",IF(H11&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -2977,7 +2988,7 @@
         <x:v>09-10 휴가 추가 후 기존 09-04~11 가용일은 4일. 권장 종료 09-21로 확장한 전체 계획창의 가용일은 10일이며 잔여 공수를 뜻하지 않는다. Runtime 검증은 플랫폼·앱 인수와 연계한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R17" s="13" t="str">
-        <x:v>Baseline v3.1.18; Ticket Pack v3.1.18; GitHub #19 snapshot 2026-09-10T05:05:52Z; 사용자 2026-09-10 면접 휴가 추가 지시; Fast Tracking 일정 권장안 2026-09-10 / 사용자 재편성 요청</x:v>
+        <x:v>Baseline/Ticket Pack v3.1.18; GitHub #19; K8S PR #2 097ddb5, #3 merge 7d44afc, #4 75d476e; audit/v3.1.18/k8s-intake-20260910.json</x:v>
       </x:c>
       <x:c r="S17" s="13" t="str">
         <x:f>IF(G17="Done","Done",IF(I17="",IF(F17="P1","Deferred P1","End TBD"),IF(I17&lt;'Executive Summary'!$B$4,"Overdue",IF(H17&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5548,7 +5559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra65014fa3f164c1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff9569fd6a0f452c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14363,47 +14374,47 @@
         <x:v>https://github.com/321Team/infra-kubernetes/pull/3</x:v>
       </x:c>
       <x:c r="C24" s="67" t="str">
-        <x:v>3309866766236bbdbe20b9e2ae1d8fd6f9233bcd</x:v>
+        <x:v>7d44afc3afff4d322cb4dbeff4433d61e23e111a</x:v>
       </x:c>
       <x:c r="D24" s="67" t="str">
-        <x:v>Evidence PARTIAL</x:v>
+        <x:v>Merged; supplement PASS</x:v>
       </x:c>
       <x:c r="E24" s="67" t="str">
-        <x:v>99 queries / empty time_state; CP→Worker 0/9, Worker→LB 3/3; supplement pending</x:v>
+        <x:v>24/24 queries; time, kubelet cause and Cockpit mask verified. Runtime pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" s="67" t="str">
-        <x:v>Review status</x:v>
+        <x:v>Runtime plans</x:v>
       </x:c>
       <x:c r="B25" s="67" t="str">
-        <x:v>https://github.com/321Team/infra-kubernetes/pull/2</x:v>
+        <x:v>https://github.com/321Team/infra-kubernetes/pull/4</x:v>
       </x:c>
       <x:c r="C25" s="67" t="str">
-        <x:v>068661e076de02669170d3582f3d596d6e1a8eb3</x:v>
+        <x:v>PR #2 097ddb5 / #4 75d476e</x:v>
       </x:c>
       <x:c r="D25" s="67" t="str">
-        <x:v>Ready for review</x:v>
+        <x:v>New HEAD review pending</x:v>
       </x:c>
       <x:c r="E25" s="67" t="str">
-        <x:v>하영님 요청됨; independent approval / runtime pending</x:v>
+        <x:v>PR #2: onsite mock 37/37, inspect 115. PR #4: local mock 74. Runtime not verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" s="67" t="str">
-        <x:v>Follow-up snapshot</x:v>
+        <x:v>K8S intake</x:v>
       </x:c>
       <x:c r="B26" s="67" t="str">
-        <x:v>audit/v3.1.18/followup-20260910.json</x:v>
+        <x:v>audit/v3.1.18/k8s-intake-20260910.json</x:v>
       </x:c>
       <x:c r="C26" s="67" t="str">
         <x:v>2026-09-10</x:v>
       </x:c>
       <x:c r="D26" s="67" t="str">
-        <x:v>Issue #10 / #14</x:v>
+        <x:v>Issues #10 / #14 / #19</x:v>
       </x:c>
       <x:c r="E26" s="67" t="str">
-        <x:v>Original source-snapshot.json preserved</x:v>
+        <x:v>Original snapshots preserved; NTP, CP2 resume, final host protection and storage pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="52" customHeight="1">
@@ -15111,7 +15122,7 @@
         <x:v>수집·정리</x:v>
       </x:c>
       <x:c r="E6" s="130" t="str">
-        <x:v>Worker supplement·ICR 변경범위 정리</x:v>
+        <x:v>CP1 보호·복구·최신 inspect 준비·ICR 범위 정리</x:v>
       </x:c>
       <x:c r="F6" s="130" t="str">
         <x:v>ICR-D-NET-01-01</x:v>
@@ -15151,7 +15162,7 @@
         <x:v>리뷰·결정</x:v>
       </x:c>
       <x:c r="E7" s="131" t="str">
-        <x:v>PR #2 독립 리뷰·NTP 기준·평일 Review 일정 검토</x:v>
+        <x:v>PR #2/#4 재리뷰·NTP 기준·평일 Review 검토</x:v>
       </x:c>
       <x:c r="F7" s="131" t="str">
         <x:v>DEC-CAL-P1-01</x:v>
@@ -17248,7 +17259,7 @@
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="K6:K59">
-    <x:cfRule type="containsText" dxfId="37" priority="1" operator="containsText" text="OVERBOOKED"/>
+    <x:cfRule type="containsText" dxfId="38" priority="1" operator="containsText" text="OVERBOOKED"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: prepare v3.1.18 release finalization
</commit_message>
<xml_diff>
--- a/wbs/FDS_v3.1.18_WBS_and_Gantt_v1.0.xlsx
+++ b/wbs/FDS_v3.1.18_WBS_and_Gantt_v1.0.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R137a26d119ab4fa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R2b78cea4860f46f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R02176cc0027a4d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R4b8617fd2af240c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R3b845c23c57a46c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R279c4388cc5a4e37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R31006a1b979b4f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R09d66d5b4d934e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R0014c28a50aa4e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rcc79c89ada854c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rb87c79f96a824ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R735bf5c314ac4d2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rfca90b01225e4bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R5f9d05df07d445af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R4f3e8529c58344a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Recf9f24bc52a4f9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Rf83e5ff918d348a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R4b9886d315be4d71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="39">
+  <x:dxfs count="40">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1011,6 +1011,17 @@
         <x:color rgb="FFB4233D"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFDE3E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB4233D"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE3E7"/>
         </x:patternFill>
@@ -1266,7 +1277,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rae5a8ad124bb46de"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb60bf396596841f7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1296,7 +1307,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3d52f5ad47624164"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R812d8636bd3b431c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1554,7 +1565,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Executive Schedule Summary (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Executive Schedule Summary (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -1615,7 +1626,7 @@
         <x:v>Canonical version</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>3.1.18 CANDIDATE</x:v>
+        <x:v>3.1.18 RELEASED</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
         <x:v>G1 Target</x:v>
@@ -1982,7 +1993,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a2969211bc44256"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4740b4d0a9bc43d4"/>
 </x:worksheet>
 </file>
 
@@ -2013,7 +2024,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · WBS (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · WBS (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -2045,7 +2056,7 @@
         <x:v>Canonical</x:v>
       </x:c>
       <x:c r="D2" s="17" t="str">
-        <x:v>3.1.18 CANDIDATE / Fast Tracking</x:v>
+        <x:v>3.1.18 RELEASED / Fast Tracking</x:v>
       </x:c>
       <x:c r="E2" s="17" t="str">
         <x:v>Records</x:v>
@@ -5559,7 +5570,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff9569fd6a0f452c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7583459ed90c483c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5607,7 +5618,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Phase 1 Gantt (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Phase 1 Gantt (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -9427,7 +9438,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Phase 2 Gantt (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Phase 2 Gantt (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -12572,7 +12583,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Milestones &amp; Decision Calendar (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Milestones &amp; Decision Calendar (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -13568,7 +13579,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Risks, Assumptions &amp; Lead Decisions (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Risks, Assumptions &amp; Lead Decisions (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -13917,7 +13928,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Sources &amp; Change Log (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Sources &amp; Change Log (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -14511,7 +14522,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="79" t="str">
-        <x:v>FDS v3.1.18 · Team Availability Calendar (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.18 · Team Availability Calendar (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="79"/>
       <x:c r="C1" s="79"/>
@@ -17259,7 +17270,7 @@
     <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="K6:K59">
-    <x:cfRule type="containsText" dxfId="38" priority="1" operator="containsText" text="OVERBOOKED"/>
+    <x:cfRule type="containsText" dxfId="39" priority="1" operator="containsText" text="OVERBOOKED"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>